<commit_message>
Writing data in excel
</commit_message>
<xml_diff>
--- a/Data Driven Testing/SSLLoginExcel.xlsx
+++ b/Data Driven Testing/SSLLoginExcel.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\visual Studio Code WorkSpace\Playwright_B1\Data Driven Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C9D8BCC-7658-4670-AEDF-7D38BACF89CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47A01321-9795-4ACD-BDE6-3522B9F71140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="3">
   <si>
     <t>https://shoppersstack.com/</t>
   </si>
@@ -389,4 +390,34 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{122F7958-6126-4E45-B9D9-A3040B91CC68}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" r:id="rId1" xr:uid="{9B2B3B46-4309-4FCC-8FEE-5BB405DC8773}"/>
+    <hyperlink ref="A2" r:id="rId2" xr:uid="{392D3A7E-5EA5-4AB9-9618-28AD1294F714}"/>
+    <hyperlink ref="A3" r:id="rId3" xr:uid="{6AB88EFD-64D9-4FC4-BF85-B50F0C9FF7EC}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>